<commit_message>
fix up showing evening stats
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B9F87A-1B92-4EAE-91F1-07CC54900F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0CC0B76-7A69-4573-A9E3-F2F621D100A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -1670,20 +1670,6 @@
 updated to reflect victory points for both your tank and friendly forces. </t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e006c Retrofit Period - Gyrostabilizer&lt;/Bold&gt; 
-&lt;InlineUIContainer&gt;&lt;Button Content='r27.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Since the refit takes at least 7 days, the date is past Nov 1st 1944, and your crew has a combined rating of 30, your crew is trained in the use of the gyrostablilizer per 
-&lt;InlineUIContainer&gt;&lt;Button Content='r27.22' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Loss of the gunner loses the Horizontal Volute Spring Suspension (HVSS) capability. Note: HVSS only appear when a tank replacement occurs, and the HVSS die roll check passes per 
-&lt;InlineUIContainer&gt;&lt;Button Content='r5.25' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Click image to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                                  &lt;InlineUIContainer&gt;&lt;Image Name='c75Hvss'  Height='80' Width='80'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;e013a Out of Main Gun Rounds&lt;/Bold&gt; 
 &lt;InlineUIContainer&gt;&lt;Button Content='r9.6' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;   
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -1704,6 +1690,20 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='Weather' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; Table.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
 Die Roll: &lt;InlineUIContainer&gt;&lt;Image Name='DieRollBlue' Height='21' Width='21' &gt; &lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e006c Retrofit Period - Gyrostabilizer&lt;/Bold&gt; 
+&lt;InlineUIContainer&gt;&lt;Button Content='r27.2' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Since the refit takes at least 7 days and your crew has a combined rating of 30, your gunner is trained in the use of the gyrostablilizer per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r27.22' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Loss of the gunner loses the Horizontal Volute Spring Suspension (HVSS) capability. Note: HVSS only appear when a tank replacement occurs, and the HVSS die roll check passes per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r5.25' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. HVSS cannot appear before November 1944 and will only appear for tanks mats 11 or greater.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+Click image to continue.
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                                                  &lt;InlineUIContainer&gt;&lt;Image Name='c75Hvss'  Height='80' Width='80'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -2154,12 +2154,12 @@
         <v>194</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="180" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>193</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -2279,7 +2279,7 @@
         <v>147</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -2791,7 +2791,7 @@
         <v>115</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="60" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix issue with new members. Fix isssue with all crewmen at 10
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0CC0B76-7A69-4573-A9E3-F2F621D100A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7519132-1791-416F-B464-C8A221F238F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -1640,15 +1640,6 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e007b Crew Replacement&lt;/Bold&gt; 
-&lt;InlineUIContainer&gt;&lt;Button Content='r19.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;     
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-When you tank is knocked out, wounded crewmen are replaced automatically on the next After Action Report 
-&lt;InlineUIContainer&gt;&lt;Button Content='e006' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;.  Click image to continue.  
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                          &lt;InlineUIContainer&gt;&lt;Image Name='Ambulance3' Height='160' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;e006a Retrofit Period&lt;/Bold&gt; 
 &lt;InlineUIContainer&gt;&lt;Button Content='r27.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
@@ -1704,6 +1695,15 @@
 Click image to continue.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                                                   &lt;InlineUIContainer&gt;&lt;Image Name='c75Hvss'  Height='80' Width='80'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e007b Crew Replacement&lt;/Bold&gt; 
+&lt;InlineUIContainer&gt;&lt;Button Content='r19.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;     
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+When you tank is knocked out, wounded crewmen are replaced automatically on the next After Action Report 
+&lt;InlineUIContainer&gt;&lt;Button Content='AAR' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; with ratings automatically rolled.  Click image to continue.  
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                          &lt;InlineUIContainer&gt;&lt;Image Name='Ambulance3' Height='160' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
 </sst>
 </file>
@@ -2143,7 +2143,7 @@
         <v>191</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2159,7 +2159,7 @@
         <v>193</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -2175,7 +2175,7 @@
         <v>181</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2279,7 +2279,7 @@
         <v>147</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -2791,7 +2791,7 @@
         <v>115</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -3039,7 +3039,7 @@
         <v>97</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="165" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
1.) For e030, only reduce MG by 1/2 D instead of full D. 2.) For e029a, indicate if MG or HE causes lack of firing.
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7519132-1791-416F-B464-C8A221F238F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{159A000D-5A0F-412B-80DB-7D92A8DC042E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -1051,15 +1051,6 @@
     <t>e029a</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;Bold&gt;e029a Advancing Fire Not Allowed&lt;/Bold&gt; 
-&lt;InlineUIContainer&gt;&lt;Button Content='r4.54.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  
-&lt;InlineUIContainer&gt;&lt;Button Content='r22.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-Advancing fire is only allowed if there is an HE Gun Load per &lt;InlineUIContainer&gt;&lt;Button Content='r9.61' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. Choose image below to continue.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                                            &lt;InlineUIContainer&gt;&lt;Image Name='c44AdvanceFireDeny' Height='120' Width='120'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt; </t>
-  </si>
-  <si>
     <t>e061</t>
   </si>
   <si>
@@ -1704,6 +1695,12 @@
 &lt;InlineUIContainer&gt;&lt;Button Content='AAR' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; with ratings automatically rolled.  Click image to continue.  
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;
                           &lt;InlineUIContainer&gt;&lt;Image Name='Ambulance3' Height='160' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e029a Advancing Fire Not Allowed&lt;/Bold&gt; 
+&lt;InlineUIContainer&gt;&lt;Button Content='r4.54.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  
+&lt;InlineUIContainer&gt;&lt;Button Content='r22.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
 </sst>
 </file>
@@ -2079,7 +2076,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="225" x14ac:dyDescent="0.25">
@@ -2087,7 +2084,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="120.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2095,7 +2092,7 @@
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -2103,7 +2100,7 @@
         <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -2111,7 +2108,7 @@
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -2119,15 +2116,15 @@
         <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="210" x14ac:dyDescent="0.25">
@@ -2135,79 +2132,79 @@
         <v>13</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -2215,12 +2212,12 @@
         <v>14</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>57</v>
@@ -2231,7 +2228,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -2239,7 +2236,7 @@
         <v>16</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="180" x14ac:dyDescent="0.25">
@@ -2247,15 +2244,15 @@
         <v>17</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -2279,7 +2276,7 @@
         <v>147</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -2356,18 +2353,18 @@
     </row>
     <row r="36" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>220</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -2407,7 +2404,7 @@
         <v>37</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2426,12 +2423,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="120" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>171</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>172</v>
+        <v>255</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -2460,10 +2457,10 @@
     </row>
     <row r="49" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>198</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -2500,10 +2497,10 @@
     </row>
     <row r="54" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -2519,7 +2516,7 @@
         <v>67</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="270" x14ac:dyDescent="0.25">
@@ -2559,7 +2556,7 @@
         <v>69</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="150" x14ac:dyDescent="0.25">
@@ -2567,7 +2564,7 @@
         <v>70</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2647,7 +2644,7 @@
         <v>73</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -2703,7 +2700,7 @@
         <v>65</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="75" x14ac:dyDescent="0.25">
@@ -2711,7 +2708,7 @@
         <v>138</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2719,7 +2716,7 @@
         <v>139</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2727,7 +2724,7 @@
         <v>140</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2740,10 +2737,10 @@
     </row>
     <row r="84" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B84" s="2" t="s">
         <v>237</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -2759,7 +2756,7 @@
         <v>136</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -2791,7 +2788,7 @@
         <v>115</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -2855,7 +2852,7 @@
         <v>148</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -2900,34 +2897,34 @@
     </row>
     <row r="104" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B107" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -2964,58 +2961,58 @@
     </row>
     <row r="112" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B113" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="B113" s="2" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B116" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="B116" s="2" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B117" s="2" t="s">
         <v>207</v>
-      </c>
-      <c r="B117" s="2" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="B118" s="2" t="s">
         <v>209</v>
-      </c>
-      <c r="B118" s="2" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -3031,7 +3028,7 @@
         <v>159</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -3039,7 +3036,7 @@
         <v>97</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="165" x14ac:dyDescent="0.25">
@@ -3047,7 +3044,7 @@
         <v>98</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="135" x14ac:dyDescent="0.25">
@@ -3087,7 +3084,7 @@
         <v>6</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="60" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix spelling errors identified by Joy
</commit_message>
<xml_diff>
--- a/DesignDocs/Events.xlsx
+++ b/DesignDocs/Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cstew\source\repos\PattonsBest\DesignDocs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{159A000D-5A0F-412B-80DB-7D92A8DC042E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B53FD1DA-B0A9-4D61-B3B2-025CDAC4150A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{89590866-6083-4176-8CBF-8C95C9BA24C2}"/>
   </bookViews>
@@ -1631,18 +1631,6 @@
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e006a Retrofit Period&lt;/Bold&gt; 
-&lt;InlineUIContainer&gt;&lt;Button Content='r27.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-During the periods on the Combat &lt;InlineUIContainer&gt;&lt;Button Content='Calendar' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
- marked Refitting, the Division is building itself back up to strength, replacing tanks, and retraining crews. 
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-During a refit period, you have the option of replacing your current tank per 
-&lt;InlineUIContainer&gt;&lt;Button Content='r24.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
-If the refit period is over 7 days, the crew goes through additional training resulting in possilbe crew rating improvements.
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
-  </si>
-  <si>
     <t xml:space="preserve">&lt;Bold&gt;e101 Evening Debriefing - Victory Point Total&lt;/Bold&gt; 
 &lt;InlineUIContainer&gt;&lt;Button Content='r4.92' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  
 &lt;InlineUIContainer&gt;&lt;Button Content='r6.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
@@ -1688,18 +1676,30 @@
                                                   &lt;InlineUIContainer&gt;&lt;Image Name='c75Hvss'  Height='80' Width='80'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
   </si>
   <si>
-    <t>&lt;Bold&gt;e007b Crew Replacement&lt;/Bold&gt; 
-&lt;InlineUIContainer&gt;&lt;Button Content='r19.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;     
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-When you tank is knocked out, wounded crewmen are replaced automatically on the next After Action Report 
-&lt;InlineUIContainer&gt;&lt;Button Content='AAR' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; with ratings automatically rolled.  Click image to continue.  
-&lt;LineBreak/&gt;&lt;LineBreak/&gt;
-                          &lt;InlineUIContainer&gt;&lt;Image Name='Ambulance3' Height='160' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
-  </si>
-  <si>
     <t>&lt;Bold&gt;e029a Advancing Fire Not Allowed&lt;/Bold&gt; 
 &lt;InlineUIContainer&gt;&lt;Button Content='r4.54.5' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;  
 &lt;InlineUIContainer&gt;&lt;Button Content='r22.1' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e007b Crew Replacement&lt;/Bold&gt; 
+&lt;InlineUIContainer&gt;&lt;Button Content='r19.3' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;     
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+When your tank is knocked out, wounded crewmen are replaced automatically on the next After Action Report 
+&lt;InlineUIContainer&gt;&lt;Button Content='AAR' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; with ratings automatically rolled.  Click image to continue.  
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+                          &lt;InlineUIContainer&gt;&lt;Image Name='Ambulance3' Height='160' Width='300'&gt;&lt;/Image&gt;&lt;/InlineUIContainer&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Bold&gt;e006a Retrofit Period&lt;/Bold&gt; 
+&lt;InlineUIContainer&gt;&lt;Button Content='r27.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt; 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+During the periods on the Combat &lt;InlineUIContainer&gt;&lt;Button Content='Calendar' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;
+ marked Refitting, the Division is building itself back up to strength, replacing tanks, and retraining crews. 
+&lt;LineBreak/&gt;&lt;LineBreak/&gt;
+During a refit period, you have the option of replacing your current tank per 
+&lt;InlineUIContainer&gt;&lt;Button Content='r24.0' FontFamily='Courier New'  FontSize='12'&gt;&lt;/Button&gt;&lt;/InlineUIContainer&gt;. 
+If the refit period is over 7 days, the crew goes through additional training resulting in possible crew rating improvements.
 &lt;LineBreak/&gt;&lt;LineBreak/&gt;</t>
   </si>
 </sst>
@@ -2140,7 +2140,7 @@
         <v>190</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="90" x14ac:dyDescent="0.25">
@@ -2156,7 +2156,7 @@
         <v>192</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -2276,7 +2276,7 @@
         <v>147</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="120" x14ac:dyDescent="0.25">
@@ -2428,7 +2428,7 @@
         <v>171</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="105" x14ac:dyDescent="0.25">
@@ -2788,7 +2788,7 @@
         <v>115</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="60" x14ac:dyDescent="0.25">
@@ -3036,7 +3036,7 @@
         <v>97</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="165" x14ac:dyDescent="0.25">

</xml_diff>